<commit_message>
Parts on first assembly.
</commit_message>
<xml_diff>
--- a/Capstan Drive Hopper BOM.xlsx
+++ b/Capstan Drive Hopper BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jtper\Documents\Summer_UROP\hopping_robot\CAD\Parts\Capstan-Drive-Hopper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF15C923-EC31-4F47-AF00-281B59B3F54B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0BA30D-A67B-4849-B1A9-13DBB939EA89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18732" yWindow="9576" windowWidth="18840" windowHeight="13176" xr2:uid="{524B48DA-7D71-4E1E-A711-D21F403C7411}"/>
+    <workbookView xWindow="-18792" yWindow="9516" windowWidth="18960" windowHeight="13296" xr2:uid="{524B48DA-7D71-4E1E-A711-D21F403C7411}"/>
   </bookViews>
   <sheets>
     <sheet name="Hopper BOM" sheetId="2" r:id="rId1"/>
@@ -343,9 +343,6 @@
     <t>Mastrant M2 Premium (100M drum)</t>
   </si>
   <si>
-    <t>15x24x7mm Thin Section Bearing</t>
-  </si>
-  <si>
     <t>1.46-2.88</t>
   </si>
   <si>
@@ -398,6 +395,9 @@
   </si>
   <si>
     <t>Get as expedited shipping such that it will get here early next week</t>
+  </si>
+  <si>
+    <t>15x24x5mm Thin Section Bearing</t>
   </si>
 </sst>
 </file>
@@ -925,7 +925,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
@@ -964,7 +964,35 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -985,50 +1013,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1365,28 +1355,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29B155AF-2391-442A-B596-D0A4A918F669}">
   <dimension ref="A1:I37"/>
-  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="30.703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.87890625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5859375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.29296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.87890625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="55.52734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="55.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B1" s="45" t="s">
+    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1406,562 +1396,543 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="14.35" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="64" t="s">
+    <row r="3" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="51" t="s">
+      <c r="B3" s="7" t="s">
         <v>96</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="63">
+      <c r="D3">
         <v>107.9</v>
       </c>
-      <c r="E3" s="63">
-        <v>2</v>
-      </c>
-      <c r="F3" s="63">
-        <v>2</v>
-      </c>
-      <c r="G3" s="52">
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3" s="38">
         <f>F3*D3</f>
         <v>215.8</v>
       </c>
-      <c r="H3" s="53"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A4" s="64"/>
-      <c r="B4" s="55" t="s">
+      <c r="H3" s="39"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="50"/>
+      <c r="B4" s="9" t="s">
         <v>97</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="63">
+      <c r="D4">
         <v>130.82</v>
       </c>
-      <c r="E4" s="63">
-        <v>2</v>
-      </c>
-      <c r="F4" s="63">
-        <v>2</v>
-      </c>
-      <c r="G4" s="56">
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4" s="8">
         <f>F4*D4</f>
         <v>261.64</v>
       </c>
-      <c r="H4" s="68" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A5" s="64"/>
-      <c r="B5" s="66" t="s">
-        <v>115</v>
-      </c>
-      <c r="C5" s="65"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="65"/>
-      <c r="G5" s="67">
+      <c r="H4" s="45" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="50"/>
+      <c r="B5" s="51" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="44">
         <f>SUM(G3:G4)</f>
         <v>477.44</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A6" s="64"/>
-      <c r="B6" s="55"/>
-      <c r="C6" s="63"/>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="53"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A7" s="64"/>
-      <c r="B7" s="55" t="s">
-        <v>100</v>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="50"/>
+      <c r="B6" s="9"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="39"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="50"/>
+      <c r="B7" s="9" t="s">
+        <v>118</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="63" t="s">
-        <v>101</v>
-      </c>
-      <c r="E7" s="63">
+      <c r="D7" t="s">
+        <v>100</v>
+      </c>
+      <c r="E7">
         <v>3</v>
       </c>
-      <c r="F7" s="63">
+      <c r="F7">
         <v>3</v>
       </c>
-      <c r="G7" s="56">
+      <c r="G7" s="8">
         <v>7.02</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A8" s="64"/>
-      <c r="B8" s="55" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="50"/>
+      <c r="B8" s="9" t="s">
         <v>29</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="D8" s="63">
+        <v>112</v>
+      </c>
+      <c r="D8">
         <v>6.49</v>
       </c>
-      <c r="E8" s="63">
+      <c r="E8">
         <v>4</v>
       </c>
-      <c r="F8" s="63">
+      <c r="F8">
         <v>4</v>
       </c>
-      <c r="G8" s="56">
+      <c r="G8" s="8">
         <f>F8*D8</f>
         <v>25.96</v>
       </c>
-      <c r="H8" s="62" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A9" s="64"/>
-      <c r="B9" s="55" t="s">
+      <c r="H8" s="43" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="50"/>
+      <c r="B9" s="9" t="s">
         <v>99</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D9" s="63">
+      <c r="D9">
         <v>39.950000000000003</v>
       </c>
-      <c r="E9" s="63">
+      <c r="E9">
         <v>1</v>
       </c>
-      <c r="F9" s="63">
+      <c r="F9">
         <v>1</v>
       </c>
-      <c r="G9" s="56">
+      <c r="G9" s="8">
         <v>39.950000000000003</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A10" s="64"/>
-      <c r="B10" s="55"/>
-      <c r="C10" s="63"/>
-      <c r="D10" s="63"/>
-      <c r="E10" s="63"/>
-      <c r="F10" s="63"/>
-      <c r="G10" s="56"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A11" s="64"/>
-      <c r="B11" s="55" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="50"/>
+      <c r="B10" s="9"/>
+      <c r="G10" s="8"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="50"/>
+      <c r="B11" s="9" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="63" t="s">
+      <c r="D11" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="63">
+      <c r="E11">
         <v>8</v>
       </c>
-      <c r="F11" s="63">
+      <c r="F11">
         <v>12</v>
       </c>
-      <c r="G11" s="56">
+      <c r="G11" s="8">
         <v>2.04</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A12" s="64"/>
-      <c r="B12" s="55" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="50"/>
+      <c r="B12" s="9" t="s">
         <v>14</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="63" t="s">
+      <c r="D12" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="63">
+      <c r="E12">
         <v>8</v>
       </c>
-      <c r="F12" s="63">
+      <c r="F12">
         <v>12</v>
       </c>
-      <c r="G12" s="56">
+      <c r="G12" s="8">
         <v>1.68</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A13" s="64"/>
-      <c r="B13" s="55" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="50"/>
+      <c r="B13" s="9" t="s">
         <v>54</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="D13" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="63">
+      <c r="E13">
         <v>8</v>
       </c>
-      <c r="F13" s="63">
+      <c r="F13">
         <v>12</v>
       </c>
-      <c r="G13" s="56">
+      <c r="G13" s="8">
         <v>9.24</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A14" s="64"/>
-      <c r="B14" s="55"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="63"/>
-      <c r="G14" s="56"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A15" s="64"/>
-      <c r="B15" s="55" t="s">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="50"/>
+      <c r="B14" s="9"/>
+      <c r="G14" s="8"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="50"/>
+      <c r="B15" s="9" t="s">
         <v>4</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="63" t="s">
+      <c r="D15" t="s">
         <v>6</v>
       </c>
-      <c r="E15" s="63">
+      <c r="E15">
         <v>8</v>
       </c>
-      <c r="F15" s="63">
+      <c r="F15">
         <v>12</v>
       </c>
-      <c r="G15" s="56">
+      <c r="G15" s="8">
         <v>2.4</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A16" s="64"/>
-      <c r="B16" s="55" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="50"/>
+      <c r="B16" s="9" t="s">
         <v>10</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="63" t="s">
+      <c r="D16" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="63">
+      <c r="E16">
         <v>8</v>
       </c>
-      <c r="F16" s="63">
+      <c r="F16">
         <v>12</v>
       </c>
-      <c r="G16" s="56">
+      <c r="G16" s="8">
         <v>1.44</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A17" s="64"/>
-      <c r="B17" s="55" t="s">
-        <v>105</v>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="50"/>
+      <c r="B17" s="9" t="s">
+        <v>104</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D17" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="E17" s="63">
-        <v>2</v>
-      </c>
-      <c r="F17" s="63">
-        <v>2</v>
-      </c>
-      <c r="G17" s="56">
+      <c r="D17" t="s">
+        <v>105</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17">
+        <v>2</v>
+      </c>
+      <c r="G17" s="8">
         <f>F17*0.5</f>
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A18" s="64"/>
-      <c r="B18" s="55" t="s">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="50"/>
+      <c r="B18" s="9" t="s">
         <v>27</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="63" t="s">
+      <c r="D18" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="63">
+      <c r="E18">
         <v>8</v>
       </c>
-      <c r="F18" s="63">
+      <c r="F18">
         <v>12</v>
       </c>
-      <c r="G18" s="56">
+      <c r="G18" s="8">
         <v>1.56</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A19" s="64"/>
-      <c r="B19" s="55"/>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="50"/>
+      <c r="B19" s="9"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="63"/>
-      <c r="E19" s="63"/>
-      <c r="F19" s="63"/>
-      <c r="G19" s="56"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A20" s="64"/>
-      <c r="B20" s="55" t="s">
-        <v>111</v>
+      <c r="G19" s="8"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="50"/>
+      <c r="B20" s="9" t="s">
+        <v>110</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D20" s="63" t="s">
-        <v>112</v>
-      </c>
-      <c r="E20" s="63">
+      <c r="D20" t="s">
+        <v>111</v>
+      </c>
+      <c r="E20">
         <v>8</v>
       </c>
-      <c r="F20" s="63">
+      <c r="F20">
         <v>12</v>
       </c>
-      <c r="G20" s="56">
+      <c r="G20" s="8">
         <f>F20*0.16</f>
         <v>1.92</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A21" s="64"/>
-      <c r="B21" s="55" t="s">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="50"/>
+      <c r="B21" s="9" t="s">
         <v>22</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D21" s="63" t="s">
+      <c r="D21" t="s">
         <v>11</v>
       </c>
-      <c r="E21" s="63">
+      <c r="E21">
         <v>11</v>
       </c>
-      <c r="F21" s="63">
+      <c r="F21">
         <v>12</v>
       </c>
-      <c r="G21" s="56">
+      <c r="G21" s="8">
         <f>F21*0.12</f>
         <v>1.44</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A22" s="64"/>
-      <c r="B22" s="55" t="s">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="50"/>
+      <c r="B22" s="9" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="63" t="s">
+      <c r="D22" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="63">
+      <c r="E22">
         <v>8</v>
       </c>
-      <c r="F22" s="63">
+      <c r="F22">
         <v>8</v>
       </c>
-      <c r="G22" s="56">
+      <c r="G22" s="8">
         <f>F22*0.33</f>
         <v>2.64</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A23" s="64"/>
-      <c r="B23" s="55" t="s">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="50"/>
+      <c r="B23" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D23" s="63" t="s">
+      <c r="D23" t="s">
         <v>34</v>
       </c>
-      <c r="E23" s="63">
+      <c r="E23">
         <v>3</v>
       </c>
-      <c r="F23" s="63">
+      <c r="F23">
         <v>4</v>
       </c>
-      <c r="G23" s="56">
+      <c r="G23" s="8">
         <v>1.48</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A24" s="64"/>
-      <c r="B24" s="55" t="s">
-        <v>102</v>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="50"/>
+      <c r="B24" s="9" t="s">
+        <v>101</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D24" s="63" t="s">
-        <v>103</v>
-      </c>
-      <c r="E24" s="63">
+      <c r="D24" t="s">
+        <v>102</v>
+      </c>
+      <c r="E24">
         <v>1</v>
       </c>
-      <c r="F24" s="63">
-        <v>2</v>
-      </c>
-      <c r="G24" s="56">
+      <c r="F24">
+        <v>2</v>
+      </c>
+      <c r="G24" s="8">
         <f>0.61*2</f>
         <v>1.22</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A25" s="64"/>
-      <c r="B25" s="55" t="s">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="50"/>
+      <c r="B25" s="9" t="s">
         <v>21</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D25" s="63" t="s">
-        <v>104</v>
-      </c>
-      <c r="E25" s="63">
+      <c r="D25" t="s">
+        <v>103</v>
+      </c>
+      <c r="E25">
         <v>1</v>
       </c>
-      <c r="F25" s="63">
-        <v>2</v>
-      </c>
-      <c r="G25" s="56">
+      <c r="F25">
+        <v>2</v>
+      </c>
+      <c r="G25" s="8">
         <f>2*3.02</f>
         <v>6.04</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A26" s="64"/>
-      <c r="B26" s="55"/>
-      <c r="C26" s="63"/>
-      <c r="D26" s="63"/>
-      <c r="E26" s="63"/>
-      <c r="F26" s="63"/>
-      <c r="G26" s="56"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A27" s="64"/>
-      <c r="B27" s="55" t="s">
-        <v>107</v>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="50"/>
+      <c r="B26" s="9"/>
+      <c r="G26" s="8"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="50"/>
+      <c r="B27" s="9" t="s">
+        <v>106</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D27" s="63" t="s">
-        <v>108</v>
-      </c>
-      <c r="E27" s="63">
+      <c r="D27" t="s">
+        <v>107</v>
+      </c>
+      <c r="E27">
         <v>4</v>
       </c>
-      <c r="F27" s="63">
+      <c r="F27">
         <v>4</v>
       </c>
-      <c r="G27" s="56">
+      <c r="G27" s="8">
         <f>F27*0.28</f>
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A28" s="64"/>
-      <c r="B28" s="55" t="s">
-        <v>109</v>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="50"/>
+      <c r="B28" s="9" t="s">
+        <v>108</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D28" s="63" t="s">
-        <v>110</v>
-      </c>
-      <c r="E28" s="63">
+      <c r="D28" t="s">
+        <v>109</v>
+      </c>
+      <c r="E28">
         <v>4</v>
       </c>
-      <c r="F28" s="63">
+      <c r="F28">
         <v>4</v>
       </c>
-      <c r="G28" s="56">
+      <c r="G28" s="8">
         <f>F28*1.38</f>
         <v>5.52</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A29" s="64"/>
-      <c r="B29" s="57" t="s">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="50"/>
+      <c r="B29" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C29" s="58" t="s">
+      <c r="C29" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="59" t="s">
+      <c r="D29" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="E29" s="59">
+      <c r="E29" s="42">
         <v>4</v>
       </c>
-      <c r="F29" s="59">
+      <c r="F29" s="42">
         <v>4</v>
       </c>
-      <c r="G29" s="60">
+      <c r="G29" s="16">
         <v>1.6</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A30" s="64"/>
-      <c r="B30" s="66" t="s">
-        <v>116</v>
-      </c>
-      <c r="C30" s="65"/>
-      <c r="D30" s="65"/>
-      <c r="E30" s="65"/>
-      <c r="F30" s="65"/>
-      <c r="G30" s="56">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="50"/>
+      <c r="B30" s="51" t="s">
+        <v>115</v>
+      </c>
+      <c r="C30" s="52"/>
+      <c r="D30" s="52"/>
+      <c r="E30" s="52"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="8">
         <f>SUM(G7:G29)</f>
         <v>115.27000000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="64"/>
-      <c r="B31" s="48" t="s">
+    <row r="31" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="50"/>
+      <c r="B31" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="C31" s="49"/>
-      <c r="D31" s="49"/>
-      <c r="E31" s="49"/>
-      <c r="F31" s="50"/>
+      <c r="C31" s="48"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="48"/>
+      <c r="F31" s="49"/>
       <c r="G31" s="17">
         <f>G5+G30</f>
         <v>592.71</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A32" s="54"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A33" s="54"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="40"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="40"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I37">
         <v>10.25</v>
       </c>
@@ -2004,16 +1975,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6D53BBB-A303-4DD5-B9D0-47E29E885140}">
   <dimension ref="B2:I16"/>
-  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.5">
-      <c r="B2" s="61" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="4" spans="2:9" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.5">
-      <c r="B5" s="46" t="s">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="39" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B5" s="50" t="s">
         <v>37</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -2038,8 +2009,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.5">
-      <c r="B6" s="47"/>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="59"/>
       <c r="C6" s="7" t="s">
         <v>16</v>
       </c>
@@ -2063,8 +2034,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.5">
-      <c r="B7" s="47"/>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="59"/>
       <c r="C7" s="9" t="s">
         <v>17</v>
       </c>
@@ -2085,8 +2056,8 @@
         <v>0.39237000000000005</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.5">
-      <c r="B8" s="47"/>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B8" s="59"/>
       <c r="C8" s="9" t="s">
         <v>20</v>
       </c>
@@ -2107,8 +2078,8 @@
         <v>1.0093175000000001</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.5">
-      <c r="B9" s="47"/>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="59"/>
       <c r="C9" s="9" t="s">
         <v>23</v>
       </c>
@@ -2129,8 +2100,8 @@
         <v>0.2895625</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.5">
-      <c r="B10" s="47"/>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="59"/>
       <c r="C10" s="18" t="s">
         <v>24</v>
       </c>
@@ -2148,8 +2119,8 @@
       </c>
       <c r="H10" s="19"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.5">
-      <c r="B11" s="47"/>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="59"/>
       <c r="C11" s="9" t="s">
         <v>28</v>
       </c>
@@ -2170,8 +2141,8 @@
         <v>3.5342000000000002</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.5">
-      <c r="B12" s="47"/>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="59"/>
       <c r="C12" s="15" t="s">
         <v>32</v>
       </c>
@@ -2192,40 +2163,40 @@
         <v>1.19638</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="C13" s="41" t="s">
+    <row r="13" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="42"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
+      <c r="D13" s="56"/>
+      <c r="E13" s="56"/>
+      <c r="F13" s="56"/>
+      <c r="G13" s="56"/>
       <c r="H13" s="17">
         <f>SUM(H6:H12)</f>
         <v>9.8350799999999996</v>
       </c>
     </row>
-    <row r="14" spans="2:9" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.5">
-      <c r="C15" s="39" t="s">
+    <row r="14" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C15" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="43">
+      <c r="D15" s="54"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="54"/>
+      <c r="G15" s="54"/>
+      <c r="H15" s="57">
         <f>'Hopper BOM'!G31 + H13</f>
         <v>602.54507999999998</v>
       </c>
     </row>
-    <row r="16" spans="2:9" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="C16" s="41"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="44"/>
+    <row r="16" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="55"/>
+      <c r="D16" s="56"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="56"/>
+      <c r="G16" s="56"/>
+      <c r="H16" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2241,42 +2212,42 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D6818B9-BC2D-452B-A586-31298C2D30C6}">
   <dimension ref="A1:R27"/>
-  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.29296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.1171875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5859375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.29296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.87890625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="20" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="16.29296875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.1171875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.5859375" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B1" s="38" t="s">
+    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="60" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="J1" s="38" t="s">
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="J1" s="60" t="s">
         <v>57</v>
       </c>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
-      <c r="N1" s="38"/>
-      <c r="O1" s="38"/>
-    </row>
-    <row r="2" spans="1:18" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+    </row>
+    <row r="2" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
@@ -2320,7 +2291,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>51</v>
       </c>
@@ -2368,7 +2339,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B4" s="9" t="s">
         <v>52</v>
       </c>
@@ -2410,7 +2381,7 @@
         <v>8.5267007330044891</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B5" s="9" t="s">
         <v>67</v>
       </c>
@@ -2452,7 +2423,7 @@
         <v>10.845272550690581</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
         <v>68</v>
       </c>
@@ -2497,7 +2468,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
         <v>71</v>
       </c>
@@ -2542,7 +2513,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="10" t="s">
         <v>74</v>
       </c>
@@ -2588,8 +2559,8 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B10" s="24" t="s">
         <v>83</v>
       </c>
@@ -2632,7 +2603,7 @@
         <v>5.8946275219220503</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
         <v>76</v>
       </c>
@@ -2674,7 +2645,7 @@
         <v>6.5826952565581704</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B12" s="9" t="s">
         <v>77</v>
       </c>
@@ -2716,7 +2687,7 @@
         <v>7.2815987035507659</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>78</v>
       </c>
@@ -2759,7 +2730,7 @@
       </c>
       <c r="R13" s="1"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>81</v>
       </c>
@@ -2805,7 +2776,7 @@
       </c>
       <c r="R14" s="1"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
         <v>80</v>
       </c>
@@ -2851,7 +2822,7 @@
       </c>
       <c r="R15" s="1"/>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
         <v>79</v>
       </c>
@@ -2897,7 +2868,7 @@
       </c>
       <c r="R16" s="1"/>
     </row>
-    <row r="17" spans="2:18" x14ac:dyDescent="0.5">
+    <row r="17" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B17" s="37" t="s">
         <v>96</v>
       </c>
@@ -2943,7 +2914,7 @@
       </c>
       <c r="R17" s="1"/>
     </row>
-    <row r="18" spans="2:18" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="9" t="s">
         <v>84</v>
       </c>
@@ -2989,7 +2960,7 @@
       </c>
       <c r="R18" s="1"/>
     </row>
-    <row r="19" spans="2:18" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="9" t="s">
         <v>82</v>
       </c>
@@ -3037,7 +3008,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="20" spans="2:18" x14ac:dyDescent="0.5">
+    <row r="20" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B20" s="9" t="s">
         <v>90</v>
       </c>
@@ -3083,7 +3054,7 @@
       </c>
       <c r="R20" s="1"/>
     </row>
-    <row r="21" spans="2:18" x14ac:dyDescent="0.5">
+    <row r="21" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B21" s="9" t="s">
         <v>87</v>
       </c>
@@ -3128,7 +3099,7 @@
         <v>6.4488756161910832</v>
       </c>
     </row>
-    <row r="22" spans="2:18" x14ac:dyDescent="0.5">
+    <row r="22" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B22" s="9" t="s">
         <v>88</v>
       </c>
@@ -3174,7 +3145,7 @@
       </c>
       <c r="R22" s="1"/>
     </row>
-    <row r="23" spans="2:18" x14ac:dyDescent="0.5">
+    <row r="23" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B23" s="9" t="s">
         <v>89</v>
       </c>
@@ -3220,7 +3191,7 @@
       </c>
       <c r="R23" s="1"/>
     </row>
-    <row r="24" spans="2:18" x14ac:dyDescent="0.5">
+    <row r="24" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B24" s="9" t="s">
         <v>86</v>
       </c>
@@ -3266,7 +3237,7 @@
       </c>
       <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="2:18" x14ac:dyDescent="0.5">
+    <row r="25" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B25" s="37" t="s">
         <v>85</v>
       </c>
@@ -3312,7 +3283,7 @@
       </c>
       <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="2:18" x14ac:dyDescent="0.5">
+    <row r="26" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B26" s="9" t="s">
         <v>66</v>
       </c>
@@ -3355,7 +3326,7 @@
       </c>
       <c r="R26" s="1"/>
     </row>
-    <row r="27" spans="2:18" ht="14.7" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="10" t="s">
         <v>65</v>
       </c>

</xml_diff>

<commit_message>
Updated BOM at project end.
</commit_message>
<xml_diff>
--- a/Capstan Drive Hopper BOM.xlsx
+++ b/Capstan Drive Hopper BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jtper\Documents\Summer_UROP\hopping_robot\CAD\Parts\Capstan-Drive-Hopper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0BA30D-A67B-4849-B1A9-13DBB939EA89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D21D31-39F4-4BA3-8858-ACF333312C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18792" yWindow="9516" windowWidth="18960" windowHeight="13296" xr2:uid="{524B48DA-7D71-4E1E-A711-D21F403C7411}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="21705" xr2:uid="{524B48DA-7D71-4E1E-A711-D21F403C7411}"/>
   </bookViews>
   <sheets>
     <sheet name="Hopper BOM" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="120">
   <si>
     <t>Part Name</t>
   </si>
@@ -382,9 +382,6 @@
     <t>Amazon</t>
   </si>
   <si>
-    <t>If this is not available on Amazon Business please  let me know ASAP</t>
-  </si>
-  <si>
     <t>Big-ticket items subtotal / £</t>
   </si>
   <si>
@@ -394,10 +391,16 @@
     <t>IGNORE FOR NOW</t>
   </si>
   <si>
-    <t>Get as expedited shipping such that it will get here early next week</t>
-  </si>
-  <si>
     <t>15x24x5mm Thin Section Bearing</t>
+  </si>
+  <si>
+    <t>mjcanfd-usb-1x USB--CAN Interface</t>
+  </si>
+  <si>
+    <t>GENSACE 2200mAh 6S Battery</t>
+  </si>
+  <si>
+    <t>Ultra Power Smart Charger</t>
   </si>
 </sst>
 </file>
@@ -925,7 +928,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
@@ -971,7 +974,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1019,6 +1021,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1354,27 +1359,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29B155AF-2391-442A-B596-D0A4A918F669}">
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="55.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
@@ -1397,7 +1402,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="49" t="s">
         <v>36</v>
       </c>
       <c r="B3" s="7" t="s">
@@ -1406,13 +1411,13 @@
       <c r="C3" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="60">
         <v>107.9</v>
       </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3">
+      <c r="E3" s="60">
+        <v>2</v>
+      </c>
+      <c r="F3" s="60">
         <v>2</v>
       </c>
       <c r="G3" s="38">
@@ -1421,552 +1426,634 @@
       </c>
       <c r="H3" s="39"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="50"/>
+    <row r="4" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="49"/>
       <c r="B4" s="9" t="s">
         <v>97</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="60">
         <v>130.82</v>
       </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="F4">
+      <c r="E4" s="60">
+        <v>2</v>
+      </c>
+      <c r="F4" s="60">
         <v>2</v>
       </c>
       <c r="G4" s="8">
         <f>F4*D4</f>
         <v>261.64</v>
       </c>
-      <c r="H4" s="45" t="s">
+      <c r="H4" s="39"/>
+    </row>
+    <row r="5" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="49"/>
+      <c r="B5" s="9" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="50"/>
-      <c r="B5" s="51" t="s">
-        <v>114</v>
-      </c>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="44">
-        <f>SUM(G3:G4)</f>
-        <v>477.44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="50"/>
-      <c r="B6" s="9"/>
-      <c r="G6" s="8"/>
+      <c r="C5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="60">
+        <v>28.96</v>
+      </c>
+      <c r="E5" s="60">
+        <v>1</v>
+      </c>
+      <c r="F5" s="60">
+        <v>1</v>
+      </c>
+      <c r="G5" s="8">
+        <f t="shared" ref="G5:G7" si="0">F5*D5</f>
+        <v>28.96</v>
+      </c>
+      <c r="H5" s="39"/>
+    </row>
+    <row r="6" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="49"/>
+      <c r="B6" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="62">
+        <v>52.99</v>
+      </c>
+      <c r="E6" s="62">
+        <v>2</v>
+      </c>
+      <c r="F6" s="62">
+        <v>2</v>
+      </c>
+      <c r="G6" s="8">
+        <f t="shared" si="0"/>
+        <v>105.98</v>
+      </c>
       <c r="H6" s="39"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="50"/>
-      <c r="B7" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="A7" s="49"/>
+      <c r="B7" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="62">
+        <v>112.99</v>
+      </c>
+      <c r="E7" s="62">
+        <v>1</v>
+      </c>
+      <c r="F7" s="62">
+        <v>1</v>
+      </c>
+      <c r="G7" s="8">
+        <f t="shared" si="0"/>
+        <v>112.99</v>
+      </c>
+      <c r="H7" s="44"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="49"/>
+      <c r="B8" s="50" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="51"/>
+      <c r="D8" s="51"/>
+      <c r="E8" s="51"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="43">
+        <f>SUM(G3:G7)</f>
+        <v>725.37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="49"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="60"/>
+      <c r="D9" s="60"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="60"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="39"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="49"/>
+      <c r="B10" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D10" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="E7">
+      <c r="E10" s="60">
         <v>3</v>
       </c>
-      <c r="F7">
+      <c r="F10" s="60">
         <v>3</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G10" s="8">
         <v>7.02</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="50"/>
-      <c r="B8" s="9" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="49"/>
+      <c r="B11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D8">
+      <c r="D11" s="60">
         <v>6.49</v>
       </c>
-      <c r="E8">
+      <c r="E11" s="60">
         <v>4</v>
       </c>
-      <c r="F8">
+      <c r="F11" s="60">
         <v>4</v>
       </c>
-      <c r="G8" s="8">
-        <f>F8*D8</f>
+      <c r="G11" s="8">
+        <f>F11*D11</f>
         <v>25.96</v>
       </c>
-      <c r="H8" s="43" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="50"/>
-      <c r="B9" s="9" t="s">
+      <c r="H11" s="61"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="49"/>
+      <c r="B12" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D9">
+      <c r="D12" s="60">
         <v>39.950000000000003</v>
       </c>
-      <c r="E9">
+      <c r="E12" s="60">
         <v>1</v>
       </c>
-      <c r="F9">
+      <c r="F12" s="60">
         <v>1</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G12" s="8">
         <v>39.950000000000003</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="50"/>
-      <c r="B10" s="9"/>
-      <c r="G10" s="8"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="50"/>
-      <c r="B11" s="9" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="49"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="60"/>
+      <c r="D13" s="60"/>
+      <c r="E13" s="60"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="8"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="49"/>
+      <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D14" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="E11">
+      <c r="E14" s="60">
         <v>8</v>
       </c>
-      <c r="F11">
+      <c r="F14" s="60">
         <v>12</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G14" s="8">
         <v>2.04</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="50"/>
-      <c r="B12" s="9" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="49"/>
+      <c r="B15" s="9" t="s">
         <v>14</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12">
-        <v>8</v>
-      </c>
-      <c r="F12">
-        <v>12</v>
-      </c>
-      <c r="G12" s="8">
-        <v>1.68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="50"/>
-      <c r="B13" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13">
-        <v>8</v>
-      </c>
-      <c r="F13">
-        <v>12</v>
-      </c>
-      <c r="G13" s="8">
-        <v>9.24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="50"/>
-      <c r="B14" s="9"/>
-      <c r="G14" s="8"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="50"/>
-      <c r="B15" s="9" t="s">
-        <v>4</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15">
+      <c r="D15" s="60" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="60">
         <v>8</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="60">
         <v>12</v>
       </c>
       <c r="G15" s="8">
-        <v>2.4</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="50"/>
+      <c r="A16" s="49"/>
       <c r="B16" s="9" t="s">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16">
+      <c r="D16" s="60" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" s="60">
         <v>8</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="60">
         <v>12</v>
       </c>
       <c r="G16" s="8">
-        <v>1.44</v>
+        <v>9.24</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="50"/>
-      <c r="B17" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" t="s">
-        <v>105</v>
-      </c>
-      <c r="E17">
-        <v>2</v>
-      </c>
-      <c r="F17">
-        <v>2</v>
-      </c>
-      <c r="G17" s="8">
-        <f>F17*0.5</f>
-        <v>1</v>
-      </c>
+      <c r="A17" s="49"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="60"/>
+      <c r="G17" s="8"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="50"/>
+      <c r="A18" s="49"/>
       <c r="B18" s="9" t="s">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D18" t="s">
-        <v>26</v>
-      </c>
-      <c r="E18">
+      <c r="D18" s="60" t="s">
+        <v>6</v>
+      </c>
+      <c r="E18" s="60">
         <v>8</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="60">
         <v>12</v>
       </c>
       <c r="G18" s="8">
-        <v>1.56</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="50"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="2"/>
-      <c r="G19" s="8"/>
+      <c r="A19" s="49"/>
+      <c r="B19" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" s="60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="60">
+        <v>8</v>
+      </c>
+      <c r="F19" s="60">
+        <v>12</v>
+      </c>
+      <c r="G19" s="8">
+        <v>1.44</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="50"/>
+      <c r="A20" s="49"/>
       <c r="B20" s="9" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D20" t="s">
-        <v>111</v>
-      </c>
-      <c r="E20">
-        <v>8</v>
-      </c>
-      <c r="F20">
-        <v>12</v>
+      <c r="D20" s="60" t="s">
+        <v>105</v>
+      </c>
+      <c r="E20" s="60">
+        <v>2</v>
+      </c>
+      <c r="F20" s="60">
+        <v>2</v>
       </c>
       <c r="G20" s="8">
-        <f>F20*0.16</f>
-        <v>1.92</v>
+        <f>F20*0.5</f>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="50"/>
+      <c r="A21" s="49"/>
       <c r="B21" s="9" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D21" t="s">
-        <v>11</v>
-      </c>
-      <c r="E21">
-        <v>11</v>
-      </c>
-      <c r="F21">
+      <c r="D21" s="60" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="60">
+        <v>8</v>
+      </c>
+      <c r="F21" s="60">
         <v>12</v>
       </c>
       <c r="G21" s="8">
-        <f>F21*0.12</f>
-        <v>1.44</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="50"/>
-      <c r="B22" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" t="s">
-        <v>31</v>
-      </c>
-      <c r="E22">
-        <v>8</v>
-      </c>
-      <c r="F22">
-        <v>8</v>
-      </c>
-      <c r="G22" s="8">
-        <f>F22*0.33</f>
-        <v>2.64</v>
-      </c>
+      <c r="A22" s="49"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="60"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="60"/>
+      <c r="G22" s="8"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="50"/>
+      <c r="A23" s="49"/>
       <c r="B23" s="9" t="s">
-        <v>33</v>
+        <v>110</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D23" t="s">
-        <v>34</v>
-      </c>
-      <c r="E23">
-        <v>3</v>
-      </c>
-      <c r="F23">
-        <v>4</v>
+      <c r="D23" s="60" t="s">
+        <v>111</v>
+      </c>
+      <c r="E23" s="60">
+        <v>8</v>
+      </c>
+      <c r="F23" s="60">
+        <v>12</v>
       </c>
       <c r="G23" s="8">
-        <v>1.48</v>
+        <f>F23*0.16</f>
+        <v>1.92</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="50"/>
+      <c r="A24" s="49"/>
       <c r="B24" s="9" t="s">
-        <v>101</v>
+        <v>22</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" s="60">
+        <v>11</v>
+      </c>
+      <c r="F24" s="60">
+        <v>12</v>
+      </c>
+      <c r="G24" s="8">
+        <f>F24*0.12</f>
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="49"/>
+      <c r="B25" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="60" t="s">
+        <v>31</v>
+      </c>
+      <c r="E25" s="60">
+        <v>8</v>
+      </c>
+      <c r="F25" s="60">
+        <v>8</v>
+      </c>
+      <c r="G25" s="8">
+        <f>F25*0.33</f>
+        <v>2.64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="49"/>
+      <c r="B26" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D26" s="60" t="s">
+        <v>34</v>
+      </c>
+      <c r="E26" s="60">
+        <v>3</v>
+      </c>
+      <c r="F26" s="60">
+        <v>4</v>
+      </c>
+      <c r="G26" s="8">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="49"/>
+      <c r="B27" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="60" t="s">
         <v>102</v>
       </c>
-      <c r="E24">
+      <c r="E27" s="60">
         <v>1</v>
       </c>
-      <c r="F24">
-        <v>2</v>
-      </c>
-      <c r="G24" s="8">
+      <c r="F27" s="60">
+        <v>2</v>
+      </c>
+      <c r="G27" s="8">
         <f>0.61*2</f>
         <v>1.22</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="50"/>
-      <c r="B25" s="9" t="s">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="49"/>
+      <c r="B28" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D28" s="60" t="s">
         <v>103</v>
       </c>
-      <c r="E25">
+      <c r="E28" s="60">
         <v>1</v>
       </c>
-      <c r="F25">
-        <v>2</v>
-      </c>
-      <c r="G25" s="8">
+      <c r="F28" s="60">
+        <v>2</v>
+      </c>
+      <c r="G28" s="8">
         <f>2*3.02</f>
         <v>6.04</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="50"/>
-      <c r="B26" s="9"/>
-      <c r="G26" s="8"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="50"/>
-      <c r="B27" s="9" t="s">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="49"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="60"/>
+      <c r="D29" s="60"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="60"/>
+      <c r="G29" s="8"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="49"/>
+      <c r="B30" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D30" s="60" t="s">
         <v>107</v>
       </c>
-      <c r="E27">
+      <c r="E30" s="60">
         <v>4</v>
       </c>
-      <c r="F27">
+      <c r="F30" s="60">
         <v>4</v>
       </c>
-      <c r="G27" s="8">
-        <f>F27*0.28</f>
+      <c r="G30" s="8">
+        <f>F30*0.28</f>
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="50"/>
-      <c r="B28" s="9" t="s">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="49"/>
+      <c r="B31" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D31" s="60" t="s">
         <v>109</v>
       </c>
-      <c r="E28">
+      <c r="E31" s="60">
         <v>4</v>
       </c>
-      <c r="F28">
+      <c r="F31" s="60">
         <v>4</v>
       </c>
-      <c r="G28" s="8">
-        <f>F28*1.38</f>
+      <c r="G31" s="8">
+        <f>F31*1.38</f>
         <v>5.52</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="50"/>
-      <c r="B29" s="15" t="s">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="49"/>
+      <c r="B32" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C29" s="41" t="s">
+      <c r="C32" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="42" t="s">
+      <c r="D32" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="E29" s="42">
+      <c r="E32" s="42">
         <v>4</v>
       </c>
-      <c r="F29" s="42">
+      <c r="F32" s="42">
         <v>4</v>
       </c>
-      <c r="G29" s="16">
+      <c r="G32" s="16">
         <v>1.6</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="50"/>
-      <c r="B30" s="51" t="s">
-        <v>115</v>
-      </c>
-      <c r="C30" s="52"/>
-      <c r="D30" s="52"/>
-      <c r="E30" s="52"/>
-      <c r="F30" s="52"/>
-      <c r="G30" s="8">
-        <f>SUM(G7:G29)</f>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="49"/>
+      <c r="B33" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="C33" s="51"/>
+      <c r="D33" s="51"/>
+      <c r="E33" s="51"/>
+      <c r="F33" s="51"/>
+      <c r="G33" s="8">
+        <f>SUM(G10:G32)</f>
         <v>115.27000000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="50"/>
-      <c r="B31" s="47" t="s">
+    <row r="34" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="49"/>
+      <c r="B34" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="17">
-        <f>G5+G30</f>
-        <v>592.71</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="40"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="40"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I37">
-        <v>10.25</v>
-      </c>
+      <c r="C34" s="47"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="47"/>
+      <c r="F34" s="48"/>
+      <c r="G34" s="17">
+        <f>G8+G33</f>
+        <v>840.64</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="40"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B1:G1"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="A3:A31"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="A3:A34"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B33:F33"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{48884AE4-1669-4ABD-BF14-01D027090643}"/>
-    <hyperlink ref="C11" r:id="rId2" xr:uid="{9944BDD4-5578-4AB4-8E92-90DE11905199}"/>
-    <hyperlink ref="C12" r:id="rId3" xr:uid="{83EB5EC7-33EE-4205-8BD7-FBE9A0D25ABC}"/>
-    <hyperlink ref="C15" r:id="rId4" xr:uid="{C6E75278-0D74-4811-AD42-6BE1011BB146}"/>
-    <hyperlink ref="C16" r:id="rId5" xr:uid="{4304D289-6EEC-4DA3-9614-426EB596BC78}"/>
-    <hyperlink ref="C17" r:id="rId6" xr:uid="{00CB66CA-9102-41D8-A24A-5155ACC7EEBB}"/>
-    <hyperlink ref="C18" r:id="rId7" xr:uid="{55042FE4-BDFE-4B8D-A43D-2CA6DC73D256}"/>
-    <hyperlink ref="C21" r:id="rId8" xr:uid="{BA728EAE-0CC3-4093-8C67-398A2077C461}"/>
-    <hyperlink ref="C22" r:id="rId9" xr:uid="{8FAAC90B-A0FA-46F8-9563-7C6BA9693372}"/>
-    <hyperlink ref="C23" r:id="rId10" xr:uid="{770C89DA-ADC2-4E11-A36C-BCD0177E3DD9}"/>
-    <hyperlink ref="C29" r:id="rId11" xr:uid="{2BEBCBD4-B3BD-405D-A757-EE25E0D0D761}"/>
-    <hyperlink ref="C7" r:id="rId12" xr:uid="{9CB2A1C9-ADAD-42F4-916F-9D1C5A1E9B95}"/>
-    <hyperlink ref="C8" r:id="rId13" xr:uid="{A9FB42A2-42DC-46DA-8A8A-4FE9D78BCB6B}"/>
+    <hyperlink ref="C14" r:id="rId2" xr:uid="{9944BDD4-5578-4AB4-8E92-90DE11905199}"/>
+    <hyperlink ref="C15" r:id="rId3" xr:uid="{83EB5EC7-33EE-4205-8BD7-FBE9A0D25ABC}"/>
+    <hyperlink ref="C18" r:id="rId4" xr:uid="{C6E75278-0D74-4811-AD42-6BE1011BB146}"/>
+    <hyperlink ref="C19" r:id="rId5" xr:uid="{4304D289-6EEC-4DA3-9614-426EB596BC78}"/>
+    <hyperlink ref="C20" r:id="rId6" xr:uid="{00CB66CA-9102-41D8-A24A-5155ACC7EEBB}"/>
+    <hyperlink ref="C21" r:id="rId7" xr:uid="{55042FE4-BDFE-4B8D-A43D-2CA6DC73D256}"/>
+    <hyperlink ref="C24" r:id="rId8" xr:uid="{BA728EAE-0CC3-4093-8C67-398A2077C461}"/>
+    <hyperlink ref="C25" r:id="rId9" xr:uid="{8FAAC90B-A0FA-46F8-9563-7C6BA9693372}"/>
+    <hyperlink ref="C26" r:id="rId10" xr:uid="{770C89DA-ADC2-4E11-A36C-BCD0177E3DD9}"/>
+    <hyperlink ref="C32" r:id="rId11" xr:uid="{2BEBCBD4-B3BD-405D-A757-EE25E0D0D761}"/>
+    <hyperlink ref="C10" r:id="rId12" xr:uid="{9CB2A1C9-ADAD-42F4-916F-9D1C5A1E9B95}"/>
+    <hyperlink ref="C11" r:id="rId13" xr:uid="{A9FB42A2-42DC-46DA-8A8A-4FE9D78BCB6B}"/>
     <hyperlink ref="C3" r:id="rId14" xr:uid="{C7830AD8-9D26-403A-91F4-8EE9396C5CA4}"/>
-    <hyperlink ref="C9" r:id="rId15" xr:uid="{B70C618E-4255-424F-8B1C-206D0146C276}"/>
-    <hyperlink ref="C13" r:id="rId16" xr:uid="{60581BFB-2B5E-4065-80FD-36B32C6010FD}"/>
-    <hyperlink ref="C24" r:id="rId17" xr:uid="{82DC9C7D-06B7-487D-B04C-EFE5997062CC}"/>
-    <hyperlink ref="C25" r:id="rId18" xr:uid="{15C9350A-4F47-4DA3-8C5C-D824860EACC2}"/>
-    <hyperlink ref="C27" r:id="rId19" xr:uid="{E42AA80A-E21E-4C78-8816-EAAC349CE8E9}"/>
-    <hyperlink ref="C28" r:id="rId20" xr:uid="{C69B33D5-9E09-4CF8-883C-13E59170D440}"/>
-    <hyperlink ref="C20" r:id="rId21" xr:uid="{E0E2D8C2-1725-472F-BEAB-F5BEEE055790}"/>
+    <hyperlink ref="C12" r:id="rId15" xr:uid="{B70C618E-4255-424F-8B1C-206D0146C276}"/>
+    <hyperlink ref="C16" r:id="rId16" xr:uid="{60581BFB-2B5E-4065-80FD-36B32C6010FD}"/>
+    <hyperlink ref="C27" r:id="rId17" xr:uid="{82DC9C7D-06B7-487D-B04C-EFE5997062CC}"/>
+    <hyperlink ref="C28" r:id="rId18" xr:uid="{15C9350A-4F47-4DA3-8C5C-D824860EACC2}"/>
+    <hyperlink ref="C30" r:id="rId19" xr:uid="{E42AA80A-E21E-4C78-8816-EAAC349CE8E9}"/>
+    <hyperlink ref="C31" r:id="rId20" xr:uid="{C69B33D5-9E09-4CF8-883C-13E59170D440}"/>
+    <hyperlink ref="C23" r:id="rId21" xr:uid="{E0E2D8C2-1725-472F-BEAB-F5BEEE055790}"/>
+    <hyperlink ref="C5" r:id="rId22" xr:uid="{72A84408-526E-4CEA-8F42-036A0F970029}"/>
+    <hyperlink ref="C6" r:id="rId23" xr:uid="{574E1929-DCA9-4836-8F90-475A98091EE1}"/>
+    <hyperlink ref="C7" r:id="rId24" xr:uid="{2834647C-372C-4EA4-999B-DEE588C1AEF1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1979,12 +2066,12 @@
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="39" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="50" t="s">
+      <c r="B5" s="49" t="s">
         <v>37</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -2010,7 +2097,7 @@
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="59"/>
+      <c r="B6" s="58"/>
       <c r="C6" s="7" t="s">
         <v>16</v>
       </c>
@@ -2027,15 +2114,15 @@
         <v>1</v>
       </c>
       <c r="H6" s="8">
-        <f>'Hopper BOM'!I$37 / 1000 * E6 * G6</f>
-        <v>3.4132500000000001</v>
+        <f>'Hopper BOM'!I$40 / 1000 * E6 * G6</f>
+        <v>0</v>
       </c>
       <c r="I6" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="59"/>
+      <c r="B7" s="58"/>
       <c r="C7" s="9" t="s">
         <v>17</v>
       </c>
@@ -2052,12 +2139,12 @@
         <v>2</v>
       </c>
       <c r="H7" s="8">
-        <f>'Hopper BOM'!I$37 / 1000 * E7 * G7</f>
-        <v>0.39237000000000005</v>
+        <f>'Hopper BOM'!I$40 / 1000 * E7 * G7</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="59"/>
+      <c r="B8" s="58"/>
       <c r="C8" s="9" t="s">
         <v>20</v>
       </c>
@@ -2074,12 +2161,12 @@
         <v>1</v>
       </c>
       <c r="H8" s="8">
-        <f>'Hopper BOM'!I$37 / 1000 * E8 * G8</f>
-        <v>1.0093175000000001</v>
+        <f>'Hopper BOM'!I$40 / 1000 * E8 * G8</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="59"/>
+      <c r="B9" s="58"/>
       <c r="C9" s="9" t="s">
         <v>23</v>
       </c>
@@ -2096,12 +2183,12 @@
         <v>1</v>
       </c>
       <c r="H9" s="8">
-        <f>'Hopper BOM'!I$37 / 1000 * E9 * G9</f>
-        <v>0.2895625</v>
+        <f>'Hopper BOM'!I$40 / 1000 * E9 * G9</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="59"/>
+      <c r="B10" s="58"/>
       <c r="C10" s="18" t="s">
         <v>24</v>
       </c>
@@ -2120,7 +2207,7 @@
       <c r="H10" s="19"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="59"/>
+      <c r="B11" s="58"/>
       <c r="C11" s="9" t="s">
         <v>28</v>
       </c>
@@ -2137,12 +2224,12 @@
         <v>2</v>
       </c>
       <c r="H11" s="8">
-        <f>'Hopper BOM'!I$37 / 1000 * E11 * G11</f>
-        <v>3.5342000000000002</v>
+        <f>'Hopper BOM'!I$40 / 1000 * E11 * G11</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="59"/>
+      <c r="B12" s="58"/>
       <c r="C12" s="15" t="s">
         <v>32</v>
       </c>
@@ -2159,44 +2246,44 @@
         <v>2</v>
       </c>
       <c r="H12" s="16">
-        <f>'Hopper BOM'!I$37 / 1000 * E12 * G12</f>
-        <v>1.19638</v>
+        <f>'Hopper BOM'!I$40 / 1000 * E12 * G12</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="55" t="s">
+      <c r="C13" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="56"/>
-      <c r="E13" s="56"/>
-      <c r="F13" s="56"/>
-      <c r="G13" s="56"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="55"/>
+      <c r="F13" s="55"/>
+      <c r="G13" s="55"/>
       <c r="H13" s="17">
         <f>SUM(H6:H12)</f>
-        <v>9.8350799999999996</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C15" s="53" t="s">
+      <c r="C15" s="52" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="57">
-        <f>'Hopper BOM'!G31 + H13</f>
-        <v>602.54507999999998</v>
+      <c r="D15" s="53"/>
+      <c r="E15" s="53"/>
+      <c r="F15" s="53"/>
+      <c r="G15" s="53"/>
+      <c r="H15" s="56">
+        <f>'Hopper BOM'!G34 + H13</f>
+        <v>840.64</v>
       </c>
     </row>
     <row r="16" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="55"/>
-      <c r="D16" s="56"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="56"/>
-      <c r="H16" s="58"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="55"/>
+      <c r="E16" s="55"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="55"/>
+      <c r="H16" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2229,23 +2316,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="60" t="s">
+      <c r="B1" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="J1" s="60" t="s">
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="J1" s="59" t="s">
         <v>57</v>
       </c>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
     </row>
     <row r="2" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">

</xml_diff>